<commit_message>
fix(agentos_neo_xentral): the filter probe must send booleans lowercase too
Product.variant.isMatrix was the one filter left red, on "Invalid value: False.
Valid values are: true, false". The same defect was just fixed on the tool
surface (agent-os #16), but that does not reach here: this probe builds its own
query params rather than going through the MCP tool, so it carried its own copy
of the bare str() — str(False) is "False".

Fixing the tool alone would have left the workbook accusing the core of a filter
that works. Re-probed: Product filter 6✓/0✗, and the manifest is down to 11
failures, all of them the real ones (writes upstream accepts without persisting,
plus two price payload-shape 400s).
</commit_message>
<xml_diff>
--- a/cores/agentos_neo_xentral/verified.xlsx
+++ b/cores/agentos_neo_xentral/verified.xlsx
@@ -598,7 +598,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>verified.json zuletzt geschrieben: 2026-07-31 18:21</t>
+          <t>verified.json zuletzt geschrieben: 2026-07-31 18:38</t>
         </is>
       </c>
     </row>
@@ -1396,13 +1396,13 @@
         <v>98</v>
       </c>
       <c r="D25" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G25" t="n">
         <v>367</v>
@@ -17429,9 +17429,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>ok</t>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>offen</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -17449,7 +17449,11 @@
           <t>EAN / GTIN barcode of the product.</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>filter: no sample value on the test instance — filter not probed | search: probed with a fixture value — no sampled record carries this field</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17694,9 +17698,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>ok</t>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>offen</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -17714,7 +17718,11 @@
           <t>Manufacturer's own article number (MPN).</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>filter: no sample value on the test instance — filter not probed</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -18906,7 +18914,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>create: created prd_61991 (labelled 'VT Verify') — no delete endpoint, left in place</t>
+          <t>create: created prd_61992 (labelled 'VT Verify') — no delete endpoint, left in place</t>
         </is>
       </c>
     </row>
@@ -21499,9 +21507,9 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="G101" s="7" t="inlineStr">
-        <is>
-          <t>FEHLER</t>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
@@ -21519,11 +21527,7 @@
           <t>Whether this is the matrix (parent) product of a variant set. Filterable — the upstream key is isMatrixProduct.</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>filter: filter[variant.isMatrix] 400: Invalid value: False. Valid values are: true, false. {"matrixprodukt": ["Invalid value: False. Valid values are: true, false."]}</t>
-        </is>
-      </c>
+      <c r="K101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">

</xml_diff>